<commit_message>
Fix bad 2027 date typo in FY2026.xlsx source data
Row 78, "Tkt Recd Date" was 04.07.2027 (should be 04.07.2026), causing
Jul-2027 to appear in the month filter. Corrected the date directly in
the sheet's XML (not via openpyxl re-save, which was found to strip
cached values from the sheet's formula-driven SR No/Month columns) and
regenerated data.js.
</commit_message>
<xml_diff>
--- a/FY2026.xlsx
+++ b/FY2026.xlsx
@@ -10997,8 +10997,10 @@
         <f t="shared" ref="B78:B88" si="24">B77</f>
         <v>July</v>
       </c>
-      <c r="C78" s="5" t="s">
-        <v>239</v>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>04.07.2026</t>
+        </is>
       </c>
       <c r="F78" s="5" t="s">
         <v>240</v>

</xml_diff>